<commit_message>
atualiza dados de apoio 16092026
</commit_message>
<xml_diff>
--- a/data-raw/FFP_acoes.xlsx
+++ b/data-raw/FFP_acoes.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cecad365.sharepoint.com/sites/Splor/Documentos Compartilhados/General/@dcppn/DCPPN 2026/PPAG e LOA 2026/material de apoio/material de apoio - gerar volumes/2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\x19247953\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="13_ncr:1_{293BB599-3A1D-4D1F-A7BD-12603AC4E5D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C49F7F53-BA0F-4271-AA20-D647FF57380A}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -22,7 +21,7 @@
     <definedName name="LOCAL_MYSQL_DATE_FORMAT" hidden="1">REPT(LOCAL_YEAR_FORMAT,4)&amp;LOCAL_DATE_SEPARATOR&amp;REPT(LOCAL_MONTH_FORMAT,2)&amp;LOCAL_DATE_SEPARATOR&amp;REPT(LOCAL_DAY_FORMAT,2)&amp;" "&amp;REPT(LOCAL_HOUR_FORMAT,2)&amp;LOCAL_TIME_SEPARATOR&amp;REPT(LOCAL_MINUTE_FORMAT,2)&amp;LOCAL_TIME_SEPARATOR&amp;REPT(LOCAL_SECOND_FORMAT,2)</definedName>
     <definedName name="LOCAL_SECOND_FORMAT" hidden="1">" "</definedName>
   </definedNames>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -43,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
   <si>
     <t>COD_UO</t>
   </si>
@@ -226,12 +225,15 @@
   </si>
   <si>
     <t>BENEFÍCIOS PREVIDENCIÁRIOS - ARTEMIG</t>
+  </si>
+  <si>
+    <t>BENEFÍCIOS PREVIDENCIÁRIOS - DETRAN-MG</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -375,7 +377,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -553,12 +555,6 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -724,7 +720,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Ênfase1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -756,10 +752,10 @@
     <cellStyle name="Ênfase5" xfId="34" builtinId="45" customBuiltin="1"/>
     <cellStyle name="Ênfase6" xfId="38" builtinId="49" customBuiltin="1"/>
     <cellStyle name="Entrada" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Neutro" xfId="8" builtinId="28" customBuiltin="1"/>
+    <cellStyle name="Incorreto" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Neutra" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Nota" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Ruim" xfId="7" builtinId="27" customBuiltin="1"/>
     <cellStyle name="Saída" xfId="10" builtinId="21" customBuiltin="1"/>
     <cellStyle name="Texto de Aviso" xfId="14" builtinId="11" customBuiltin="1"/>
     <cellStyle name="Texto Explicativo" xfId="16" builtinId="53" customBuiltin="1"/>
@@ -795,7 +791,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2">
       <tableStyleElement type="wholeTable" dxfId="1"/>
       <tableStyleElement type="headerRow" dxfId="0"/>
     </tableStyle>
@@ -816,9 +812,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -856,9 +852,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -893,7 +889,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -928,7 +924,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1101,9 +1097,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:C59"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C60"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" customWidth="1"/>
@@ -1121,7 +1116,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1711</v>
       </c>
@@ -1132,7 +1127,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1721</v>
       </c>
@@ -1143,7 +1138,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2431</v>
       </c>
@@ -1154,7 +1149,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1541</v>
       </c>
@@ -1165,7 +1160,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1451</v>
       </c>
@@ -1176,7 +1171,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2441</v>
       </c>
@@ -1187,7 +1182,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>1071</v>
       </c>
@@ -1198,7 +1193,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1081</v>
       </c>
@@ -1209,7 +1204,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2071</v>
       </c>
@@ -1220,7 +1215,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>1011</v>
       </c>
@@ -1231,7 +1226,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>1031</v>
       </c>
@@ -1242,7 +1237,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>1091</v>
       </c>
@@ -1253,7 +1248,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>1051</v>
       </c>
@@ -1264,7 +1259,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>1021</v>
       </c>
@@ -1275,7 +1270,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>1441</v>
       </c>
@@ -1286,7 +1281,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>1191</v>
       </c>
@@ -1297,7 +1292,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2461</v>
       </c>
@@ -1308,7 +1303,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>1631</v>
       </c>
@@ -1319,7 +1314,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>1521</v>
       </c>
@@ -1330,7 +1325,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2311</v>
       </c>
@@ -1341,7 +1336,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2331</v>
       </c>
@@ -1352,7 +1347,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="23" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>1511</v>
       </c>
@@ -1363,7 +1358,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>1501</v>
       </c>
@@ -1374,7 +1369,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>1491</v>
       </c>
@@ -1385,7 +1380,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>1481</v>
       </c>
@@ -1396,7 +1391,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="27" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>1101</v>
       </c>
@@ -1407,7 +1402,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="28" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>1221</v>
       </c>
@@ -1418,7 +1413,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="29" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>1231</v>
       </c>
@@ -1429,7 +1424,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="30" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>1271</v>
       </c>
@@ -1440,7 +1435,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="31" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>2351</v>
       </c>
@@ -1451,7 +1446,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="32" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>1301</v>
       </c>
@@ -1462,7 +1457,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="33" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>1371</v>
       </c>
@@ -1473,7 +1468,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="34" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>1251</v>
       </c>
@@ -1484,7 +1479,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="35" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>1401</v>
       </c>
@@ -1495,7 +1490,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="36" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>2371</v>
       </c>
@@ -1506,7 +1501,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="37" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>2151</v>
       </c>
@@ -1517,7 +1512,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="38" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>2161</v>
       </c>
@@ -1528,7 +1523,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="39" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>2171</v>
       </c>
@@ -1539,7 +1534,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="40" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>2181</v>
       </c>
@@ -1550,7 +1545,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="41" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>2201</v>
       </c>
@@ -1561,7 +1556,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="42" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>2211</v>
       </c>
@@ -1572,7 +1567,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="43" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>2301</v>
       </c>
@@ -1583,7 +1578,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="44" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>2261</v>
       </c>
@@ -1594,7 +1589,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="45" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>2271</v>
       </c>
@@ -1605,7 +1600,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="46" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>2321</v>
       </c>
@@ -1616,7 +1611,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="47" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>2091</v>
       </c>
@@ -1627,7 +1622,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="48" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>2101</v>
       </c>
@@ -1638,7 +1633,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="49" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>2241</v>
       </c>
@@ -1649,7 +1644,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="50" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>2251</v>
       </c>
@@ -1660,7 +1655,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="51" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>2281</v>
       </c>
@@ -1671,7 +1666,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="52" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>2041</v>
       </c>
@@ -1682,7 +1677,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="53" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>2061</v>
       </c>
@@ -1693,7 +1688,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="54" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>2011</v>
       </c>
@@ -1704,7 +1699,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="55" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>2121</v>
       </c>
@@ -1715,7 +1710,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="56" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>2421</v>
       </c>
@@ -1726,7 +1721,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="57" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>1261</v>
       </c>
@@ -1737,7 +1732,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="58" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>4291</v>
       </c>
@@ -1759,15 +1754,19 @@
         <v>60</v>
       </c>
     </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>2481</v>
+      </c>
+      <c r="B60">
+        <v>7417</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C59" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="BENEFÍCIOS PREVIDENCIÁRIOS - ARTEMIG"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:C58">
+  <sortState ref="A4:C58">
     <sortCondition ref="B1:B58"/>
   </sortState>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -1776,7 +1775,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -1785,7 +1784,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -1794,6 +1793,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="b91e7f20-fe0a-487d-91a9-605ac1c64acf" xsi:nil="true"/>
@@ -1811,18 +1819,9 @@
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100B08D58FADB61F04EBBB4F355C06EFBED" ma:contentTypeVersion="19" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="7797dc5feb179b4da55a9ebddd321181">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6f4338ef-addb-4c87-aefe-1895241b335f" xmlns:ns3="b91e7f20-fe0a-487d-91a9-605ac1c64acf" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="90078f443198b6d5c0fd169535a443b9" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100B08D58FADB61F04EBBB4F355C06EFBED" ma:contentTypeVersion="19" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="b1e0f6055e0e9a4b9e75d6c71ee7de91">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6f4338ef-addb-4c87-aefe-1895241b335f" xmlns:ns3="b91e7f20-fe0a-487d-91a9-605ac1c64acf" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b43930f3490e4d4da1ab3f8da7df6f51" ns2:_="" ns3:_="">
     <xsd:import namespace="6f4338ef-addb-4c87-aefe-1895241b335f"/>
     <xsd:import namespace="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
     <xsd:element name="properties">
@@ -2082,17 +2081,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F7C923F2-A4FA-4B59-9477-1E7A98C0125A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
-    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B1DB9620-CC88-4257-8480-C321EF6EFF37}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -2100,21 +2088,23 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EBB7F238-CDE3-461E-8F60-E82D00978859}">
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F7C923F2-A4FA-4B59-9477-1E7A98C0125A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
-    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8581AC78-9506-4D29-B096-943C3A1421C4}"/>
 </file>
</xml_diff>

<commit_message>
Update data package at: 2026-09-22T13:03:20Z
</commit_message>
<xml_diff>
--- a/data-raw/FFP_acoes.xlsx
+++ b/data-raw/FFP_acoes.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30516"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\x19247953\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_0E52322E6C2ABBD3BBFA4E2AE92BFCD2B95CA6AE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -21,7 +22,7 @@
     <definedName name="LOCAL_MYSQL_DATE_FORMAT" hidden="1">REPT(LOCAL_YEAR_FORMAT,4)&amp;LOCAL_DATE_SEPARATOR&amp;REPT(LOCAL_MONTH_FORMAT,2)&amp;LOCAL_DATE_SEPARATOR&amp;REPT(LOCAL_DAY_FORMAT,2)&amp;" "&amp;REPT(LOCAL_HOUR_FORMAT,2)&amp;LOCAL_TIME_SEPARATOR&amp;REPT(LOCAL_MINUTE_FORMAT,2)&amp;LOCAL_TIME_SEPARATOR&amp;REPT(LOCAL_SECOND_FORMAT,2)</definedName>
     <definedName name="LOCAL_SECOND_FORMAT" hidden="1">" "</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -233,8 +234,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="19" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -720,7 +721,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Ênfase1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -752,10 +753,10 @@
     <cellStyle name="Ênfase5" xfId="34" builtinId="45" customBuiltin="1"/>
     <cellStyle name="Ênfase6" xfId="38" builtinId="49" customBuiltin="1"/>
     <cellStyle name="Entrada" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Incorreto" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Neutra" xfId="8" builtinId="28" customBuiltin="1"/>
+    <cellStyle name="Neutro" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Nota" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Ruim" xfId="7" builtinId="27" customBuiltin="1"/>
     <cellStyle name="Saída" xfId="10" builtinId="21" customBuiltin="1"/>
     <cellStyle name="Texto de Aviso" xfId="14" builtinId="11" customBuiltin="1"/>
     <cellStyle name="Texto Explicativo" xfId="16" builtinId="53" customBuiltin="1"/>
@@ -791,7 +792,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
       <tableStyleElement type="wholeTable" dxfId="1"/>
       <tableStyleElement type="headerRow" dxfId="0"/>
     </tableStyle>
@@ -807,14 +808,10 @@
 </styleSheet>
 </file>
 
-<file path=xl/namedSheetViews/namedSheetView1.xml><?xml version="1.0" encoding="utf-8"?>
-<namedSheetViews xmlns="http://schemas.microsoft.com/office/spreadsheetml/2019/namedsheetviews" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -852,9 +849,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -889,7 +886,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -924,7 +921,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1097,15 +1094,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C60"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.28515625" customWidth="1"/>
     <col min="3" max="3" width="46.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1116,7 +1113,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3">
       <c r="A2">
         <v>1711</v>
       </c>
@@ -1127,7 +1124,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3">
       <c r="A3">
         <v>1721</v>
       </c>
@@ -1138,7 +1135,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3">
       <c r="A4">
         <v>2431</v>
       </c>
@@ -1149,7 +1146,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3">
       <c r="A5">
         <v>1541</v>
       </c>
@@ -1160,7 +1157,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3">
       <c r="A6">
         <v>1451</v>
       </c>
@@ -1171,7 +1168,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3">
       <c r="A7">
         <v>2441</v>
       </c>
@@ -1182,7 +1179,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3">
       <c r="A8">
         <v>1071</v>
       </c>
@@ -1193,7 +1190,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3">
       <c r="A9">
         <v>1081</v>
       </c>
@@ -1204,7 +1201,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3">
       <c r="A10">
         <v>2071</v>
       </c>
@@ -1215,7 +1212,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3">
       <c r="A11">
         <v>1011</v>
       </c>
@@ -1226,7 +1223,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3">
       <c r="A12">
         <v>1031</v>
       </c>
@@ -1237,7 +1234,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3">
       <c r="A13">
         <v>1091</v>
       </c>
@@ -1248,7 +1245,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3">
       <c r="A14">
         <v>1051</v>
       </c>
@@ -1259,7 +1256,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3">
       <c r="A15">
         <v>1021</v>
       </c>
@@ -1270,7 +1267,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3">
       <c r="A16">
         <v>1441</v>
       </c>
@@ -1281,7 +1278,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3">
       <c r="A17">
         <v>1191</v>
       </c>
@@ -1292,7 +1289,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3">
       <c r="A18">
         <v>2461</v>
       </c>
@@ -1303,7 +1300,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3">
       <c r="A19">
         <v>1631</v>
       </c>
@@ -1314,7 +1311,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3">
       <c r="A20">
         <v>1521</v>
       </c>
@@ -1325,7 +1322,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3">
       <c r="A21">
         <v>2311</v>
       </c>
@@ -1336,7 +1333,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3">
       <c r="A22">
         <v>2331</v>
       </c>
@@ -1347,7 +1344,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3">
       <c r="A23">
         <v>1511</v>
       </c>
@@ -1358,7 +1355,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3">
       <c r="A24">
         <v>1501</v>
       </c>
@@ -1369,7 +1366,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3">
       <c r="A25">
         <v>1491</v>
       </c>
@@ -1380,7 +1377,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3">
       <c r="A26">
         <v>1481</v>
       </c>
@@ -1391,7 +1388,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3">
       <c r="A27">
         <v>1101</v>
       </c>
@@ -1402,7 +1399,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3">
       <c r="A28">
         <v>1221</v>
       </c>
@@ -1413,7 +1410,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3">
       <c r="A29">
         <v>1231</v>
       </c>
@@ -1424,7 +1421,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3">
       <c r="A30">
         <v>1271</v>
       </c>
@@ -1435,7 +1432,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3">
       <c r="A31">
         <v>2351</v>
       </c>
@@ -1446,7 +1443,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3">
       <c r="A32">
         <v>1301</v>
       </c>
@@ -1457,7 +1454,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3">
       <c r="A33">
         <v>1371</v>
       </c>
@@ -1468,7 +1465,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3">
       <c r="A34">
         <v>1251</v>
       </c>
@@ -1479,7 +1476,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3">
       <c r="A35">
         <v>1401</v>
       </c>
@@ -1490,7 +1487,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3">
       <c r="A36">
         <v>2371</v>
       </c>
@@ -1501,7 +1498,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3">
       <c r="A37">
         <v>2151</v>
       </c>
@@ -1512,7 +1509,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3">
       <c r="A38">
         <v>2161</v>
       </c>
@@ -1523,7 +1520,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3">
       <c r="A39">
         <v>2171</v>
       </c>
@@ -1534,7 +1531,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3">
       <c r="A40">
         <v>2181</v>
       </c>
@@ -1545,7 +1542,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3">
       <c r="A41">
         <v>2201</v>
       </c>
@@ -1556,7 +1553,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3">
       <c r="A42">
         <v>2211</v>
       </c>
@@ -1567,7 +1564,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3">
       <c r="A43">
         <v>2301</v>
       </c>
@@ -1578,7 +1575,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3">
       <c r="A44">
         <v>2261</v>
       </c>
@@ -1589,7 +1586,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3">
       <c r="A45">
         <v>2271</v>
       </c>
@@ -1600,7 +1597,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3">
       <c r="A46">
         <v>2321</v>
       </c>
@@ -1611,7 +1608,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3">
       <c r="A47">
         <v>2091</v>
       </c>
@@ -1622,7 +1619,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3">
       <c r="A48">
         <v>2101</v>
       </c>
@@ -1633,7 +1630,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3">
       <c r="A49">
         <v>2241</v>
       </c>
@@ -1644,7 +1641,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3">
       <c r="A50">
         <v>2251</v>
       </c>
@@ -1655,7 +1652,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3">
       <c r="A51">
         <v>2281</v>
       </c>
@@ -1666,7 +1663,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3">
       <c r="A52">
         <v>2041</v>
       </c>
@@ -1677,7 +1674,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3">
       <c r="A53">
         <v>2061</v>
       </c>
@@ -1688,7 +1685,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3">
       <c r="A54">
         <v>2011</v>
       </c>
@@ -1699,7 +1696,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3">
       <c r="A55">
         <v>2121</v>
       </c>
@@ -1710,7 +1707,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3">
       <c r="A56">
         <v>2421</v>
       </c>
@@ -1721,7 +1718,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3">
       <c r="A57">
         <v>1261</v>
       </c>
@@ -1732,7 +1729,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3">
       <c r="A58">
         <v>4291</v>
       </c>
@@ -1743,7 +1740,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3">
       <c r="A59" s="1">
         <v>2471</v>
       </c>
@@ -1754,7 +1751,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:3">
       <c r="A60">
         <v>2481</v>
       </c>
@@ -1766,7 +1763,7 @@
       </c>
     </row>
   </sheetData>
-  <sortState ref="A4:C58">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:C58">
     <sortCondition ref="B1:B58"/>
   </sortState>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -1775,51 +1772,24 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="b91e7f20-fe0a-487d-91a9-605ac1c64acf" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6f4338ef-addb-4c87-aefe-1895241b335f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <SharedWithUsers xmlns="b91e7f20-fe0a-487d-91a9-605ac1c64acf">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100B08D58FADB61F04EBBB4F355C06EFBED" ma:contentTypeVersion="19" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="b1e0f6055e0e9a4b9e75d6c71ee7de91">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6f4338ef-addb-4c87-aefe-1895241b335f" xmlns:ns3="b91e7f20-fe0a-487d-91a9-605ac1c64acf" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b43930f3490e4d4da1ab3f8da7df6f51" ns2:_="" ns3:_="">
     <xsd:import namespace="6f4338ef-addb-4c87-aefe-1895241b335f"/>
@@ -2080,31 +2050,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="b91e7f20-fe0a-487d-91a9-605ac1c64acf" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6f4338ef-addb-4c87-aefe-1895241b335f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <SharedWithUsers xmlns="b91e7f20-fe0a-487d-91a9-605ac1c64acf">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B1DB9620-CC88-4257-8480-C321EF6EFF37}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8581AC78-9506-4D29-B096-943C3A1421C4}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F7C923F2-A4FA-4B59-9477-1E7A98C0125A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B1DB9620-CC88-4257-8480-C321EF6EFF37}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8581AC78-9506-4D29-B096-943C3A1421C4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F7C923F2-A4FA-4B59-9477-1E7A98C0125A}"/>
 </file>
</xml_diff>